<commit_message>
Checkpoint: GST/TDS PRO reports, AI Document Inbox + email feeder, unified pricing
Records work built/tested across sessions but not previously committed.

- GST PRO reports: GSTR-1, GSTR-3B, HSN Summary, GSTR-2B reconciliation,
  TDS Register; GSTR-2B wallet-metered auto-pull via GSP (server-side proxy).
- AI Document Inbox: one-pass classify+extract for any incoming accounting
  document (BYOK), email feeder (IMAP read-only) + setup dialog; ledger
  hsn_code + company gst_username additive columns.
- Unified pricing.xlsx (one tab per product) + bake pipeline; RWA fed from
  the sheet; monthly prices; document_inbox feature flag.
- Version bump to 1.0.17 (Nuitka 4.1.2 / Python 3.14 build fix).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/ai_features.xlsx
+++ b/config/ai_features.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -483,6 +483,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -616,6 +617,23 @@
       <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Voice-to-voucher one-liner posting.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>document_inbox</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>byok</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Document Inbox — classify+extract any incoming doc. Heavy multi-call AI; customer's own key required.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
AHQ 1.0 release snapshot (build 1.0.30)
Bundles this cycle's UI work for the first public Accounts HQ release:
onboarding wizard (all-tier, license-aware, re-runs on upgrade), menu
redesign (sidebar/launcher) + settings hub, theme toggle, AI wallet
chip/page, desktop self-update, date-format + table sort/filter changes.
Vendor cache stays parked (VENDOR_CACHE_ENABLED=False).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/ai_features.xlsx
+++ b/config/ai_features.xlsx
@@ -509,12 +509,12 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>byok</t>
+          <t>ag_key</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Reads PDFs/images. Heavy multi-call AI — customer's own key required.</t>
+          <t>Reads PDFs/images. Built-in/wallet (AccGenie key + credits); never the customer key.</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Document Inbox — classify+extract any incoming doc. Heavy multi-call AI; customer's own key required.</t>
+          <t>Document Inbox — classify+extract any incoming doc. Heavy multi-call AI.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
WIP snapshot: save 17 days of uncommitted work (since 1.0.30)
Protective snapshot of pre-existing uncommitted working-tree state — 57
modified files (3.7k lines) + 134 new files: branding (Accounts HQ / Books
HQ logos+icons), new UI screens/nav, country support, parser/reports edits,
webapp.py web port, docs, marketing. Not authored in this commit — just
saving the user's real current code so it is recoverable, not living only in
the working folder. No file contents changed by this commit.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/config/ai_features.xlsx
+++ b/config/ai_features.xlsx
@@ -461,7 +461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -617,23 +617,6 @@
       <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Voice-to-voucher one-liner posting.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>document_inbox</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>byok</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Document Inbox — classify+extract any incoming doc. Heavy multi-call AI.</t>
         </is>
       </c>
     </row>

</xml_diff>